<commit_message>
Token & Costi 30/04/2026 — aggiornamento automatico
</commit_message>
<xml_diff>
--- a/files/token_usage.xlsx
+++ b/files/token_usage.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,44 @@
       </c>
       <c r="J5" t="n">
         <v>0.02403</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>agent:main:main</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4-6 (EU Bedrock)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" t="n">
+        <v>823</v>
+      </c>
+      <c r="F6" t="n">
+        <v>55</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>7.8e-05</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.012345</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.012423</v>
       </c>
     </row>
   </sheetData>
@@ -682,7 +720,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -692,7 +730,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>240</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4">
@@ -702,7 +740,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17800</v>
+        <v>18623</v>
       </c>
     </row>
     <row r="5">
@@ -713,7 +751,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$0.0007</t>
+          <t>$0.0008</t>
         </is>
       </c>
     </row>
@@ -725,7 +763,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$0.2670</t>
+          <t>$0.2793</t>
         </is>
       </c>
     </row>
@@ -737,7 +775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$0.2677</t>
+          <t>$0.2801</t>
         </is>
       </c>
     </row>
@@ -748,7 +786,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
@@ -758,7 +796,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4450</v>
+        <v>3725</v>
       </c>
     </row>
     <row r="10">
@@ -780,7 +818,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>